<commit_message>
Update berita 2026-08-03 09:25 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-31.xlsx
+++ b/data/berita_antara_2026-07-31.xlsx
@@ -471,33 +471,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
+          <t>Bank Neo Commerce bukukan laba bersih Rp294,85 M pada semester I 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
+          <t>Fri, 31 Jul 2026 19:20:34 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
+          <t>PT Bank Neo Commerce Tbk (BNC) membukukan laba bersih setelah pajak (profit after tax/PAT) sebesar Rp294,85 miliar pada ...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
+          <t>https://www.antaranews.com/berita/5674772/bank-neo-commerce-bukukan-laba-bersih-rp29485-m-pada-semester-i-2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/WhatsApp-Image-2026-07-31-at-17.22.56.jpeg</t>
         </is>
       </c>
     </row>
@@ -509,61 +509,61 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
+          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
+          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
+          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
+          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IIF bukukan aset Rp15 triliun dan pembiayaan baru Rp2,5 triliun</t>
+          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 23:05:50 +0700</t>
+          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PT Indonesia Infrastructure Finance (IIF) mencatat aset Rp15 triliun dan komitmen pembiayaan baru Rp2,5 triliun pada ...</t>
+          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675203/iif-bukukan-aset-rp15-triliun-dan-pembiayaan-baru-rp25-triliun</t>
+          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/B9A16C4E-32D5-4162-BA5C-89F5A5135BC8.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
         </is>
       </c>
     </row>
@@ -575,28 +575,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AAJI: PSAK 117 ubah standar laporan keuangan perusahaan asuransi</t>
+          <t>IIF bukukan aset Rp15 triliun dan pembiayaan baru Rp2,5 triliun</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 21:50:31 +0700</t>
+          <t>Fri, 31 Jul 2026 23:05:50 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Asosiasi Asuransi Jiwa Indonesia (AAJI) menyatakan penerapan Pernyataan Standar Akuntansi Keuangan (PSAK) 117 yang baru ...</t>
+          <t>PT Indonesia Infrastructure Finance (IIF) mencatat aset Rp15 triliun dan komitmen pembiayaan baru Rp2,5 triliun pada ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675049/aaji-psak-117-ubah-standar-laporan-keuangan-perusahaan-asuransi</t>
+          <t>https://www.antaranews.com/berita/5675203/iif-bukukan-aset-rp15-triliun-dan-pembiayaan-baru-rp25-triliun</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1000451545.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/B9A16C4E-32D5-4162-BA5C-89F5A5135BC8.jpeg</t>
         </is>
       </c>
     </row>
@@ -608,28 +608,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Program MBG serap anggaran Rp2,02 triliun di NTB per Juni 2026</t>
+          <t>AAJI: PSAK 117 ubah standar laporan keuangan perusahaan asuransi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 21:35:31 +0700</t>
+          <t>Fri, 31 Jul 2026 21:50:31 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kantor Wilayah Direktorat Jenderal Perbendaharaan (DPJb) Provinsi Nusa Tenggara Barat mencatat realisasi belanja negara ...</t>
+          <t>Asosiasi Asuransi Jiwa Indonesia (AAJI) menyatakan penerapan Pernyataan Standar Akuntansi Keuangan (PSAK) 117 yang baru ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675015/program-mbg-serap-anggaran-rp202-triliun-di-ntb-per-juni-2026</t>
+          <t>https://www.antaranews.com/berita/5675049/aaji-psak-117-ubah-standar-laporan-keuangan-perusahaan-asuransi</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1001426687.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1000451545.jpg</t>
         </is>
       </c>
     </row>
@@ -641,28 +641,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OJK sebut pertukaran informasi antarlembaga soal judol kian intensif</t>
+          <t>Program MBG serap anggaran Rp2,02 triliun di NTB per Juni 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 21:20:06 +0700</t>
+          <t>Fri, 31 Jul 2026 21:35:31 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) menyatakan bahwa koordinasi dan pertukaran informasi antarlembaga sebagai bagian dari ...</t>
+          <t>Kantor Wilayah Direktorat Jenderal Perbendaharaan (DPJb) Provinsi Nusa Tenggara Barat mencatat realisasi belanja negara ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674981/ojk-sebut-pertukaran-informasi-antarlembaga-soal-judol-kian-intensif</t>
+          <t>https://www.antaranews.com/berita/5675015/program-mbg-serap-anggaran-rp202-triliun-di-ntb-per-juni-2026</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/25/Nilai-transaksi-judol-setiap-tahun-240726-AP-4.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1001426687.jpg</t>
         </is>
       </c>
     </row>
@@ -674,28 +674,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ekonom: Efektivitas obligasi daerah bergantung kapasitas fiskal pemda</t>
+          <t>OJK sebut pertukaran informasi antarlembaga soal judol kian intensif</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 21:07:51 +0700</t>
+          <t>Fri, 31 Jul 2026 21:20:06 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ekonom Center of Reform on Economics (CORE) Yusuf Rendy Manilet menilai efektivitas penerbitan obligasi oleh pemerintah ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) menyatakan bahwa koordinasi dan pertukaran informasi antarlembaga sebagai bagian dari ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674956/ekonom-efektivitas-obligasi-daerah-bergantung-kapasitas-fiskal-pemda</t>
+          <t>https://www.antaranews.com/berita/5674981/ojk-sebut-pertukaran-informasi-antarlembaga-soal-judol-kian-intensif</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2020/11/13/InShot_20200910_104834146.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/25/Nilai-transaksi-judol-setiap-tahun-240726-AP-4.jpg</t>
         </is>
       </c>
     </row>
@@ -707,28 +707,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ekonom: Obligasi pemda hanya efektif untuk biayai proyek produktif</t>
+          <t>Ekonom: Efektivitas obligasi daerah bergantung kapasitas fiskal pemda</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 21:02:18 +0700</t>
+          <t>Fri, 31 Jul 2026 21:07:51 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ekonom Institute for Development of Economics and Finance (INDEF) M Rizal Taufikurahman mengatakan penerbitan obligasi ...</t>
+          <t>Ekonom Center of Reform on Economics (CORE) Yusuf Rendy Manilet menilai efektivitas penerbitan obligasi oleh pemerintah ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674952/ekonom-obligasi-pemda-hanya-efektif-untuk-biayai-proyek-produktif</t>
+          <t>https://www.antaranews.com/berita/5674956/ekonom-efektivitas-obligasi-daerah-bergantung-kapasitas-fiskal-pemda</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/01/08/20260108_141804_Chrome.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/11/13/InShot_20200910_104834146.jpg</t>
         </is>
       </c>
     </row>
@@ -740,28 +740,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OJK: Keberhasilan berantas judol tak hanya dari penurunan transaksi</t>
+          <t>Ekonom: Obligasi pemda hanya efektif untuk biayai proyek produktif</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 20:53:11 +0700</t>
+          <t>Fri, 31 Jul 2026 21:02:18 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) memandang keberhasilan pemberantasan judi online tidak hanya diukur dari penurunan ...</t>
+          <t>Ekonom Institute for Development of Economics and Finance (INDEF) M Rizal Taufikurahman mengatakan penerbitan obligasi ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674936/ojk-keberhasilan-berantas-judol-tak-hanya-dari-penurunan-transaksi</t>
+          <t>https://www.antaranews.com/berita/5674952/ekonom-obligasi-pemda-hanya-efektif-untuk-biayai-proyek-produktif</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/WhatsApp-Image-2026-07-08-at-23.55.17.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/08/20260108_141804_Chrome.jpg</t>
         </is>
       </c>
     </row>
@@ -773,28 +773,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Percepatan DBH dan TKD dinilai bisa dorong kapasitas ekonomi daerah</t>
+          <t>OJK: Keberhasilan berantas judol tak hanya dari penurunan transaksi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 19:46:08 +0700</t>
+          <t>Fri, 31 Jul 2026 20:53:11 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Kepala Ekonom Permata Bank Josua Pardede menilai rencana pemerintah mempercepat pencairan dana bagi hasil (DBH) dan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) memandang keberhasilan pemberantasan judi online tidak hanya diukur dari penurunan ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674820/percepatan-dbh-dan-tkd-dinilai-bisa-dorong-kapasitas-ekonomi-daerah</t>
+          <t>https://www.antaranews.com/berita/5674936/ojk-keberhasilan-berantas-judol-tak-hanya-dari-penurunan-transaksi</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/11/19/pardede.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/WhatsApp-Image-2026-07-08-at-23.55.17.jpeg</t>
         </is>
       </c>
     </row>
@@ -806,28 +806,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Laba konsolidasi Bank SMBC Indonesia naik 40,3 persen pada semester I</t>
+          <t>Percepatan DBH dan TKD dinilai bisa dorong kapasitas ekonomi daerah</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 19:23:27 +0700</t>
+          <t>Fri, 31 Jul 2026 19:46:08 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PT Bank SMBC Indonesia Tbk membukukan laba bersih setelah pajak konsolidasi yang diatribusikan kepada pemilik entitas ...</t>
+          <t>Kepala Ekonom Permata Bank Josua Pardede menilai rencana pemerintah mempercepat pencairan dana bagi hasil (DBH) dan ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674780/laba-konsolidasi-bank-smbc-indonesia-naik-403-persen-pada-semester-i</t>
+          <t>https://www.antaranews.com/berita/5674820/percepatan-dbh-dan-tkd-dinilai-bisa-dorong-kapasitas-ekonomi-daerah</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/Foto-2-3.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/19/pardede.jpg</t>
         </is>
       </c>
     </row>
@@ -839,28 +839,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bank Neo Commerce bukukan laba bersih Rp294,85 M pada semester I 2026</t>
+          <t>Laba konsolidasi Bank SMBC Indonesia naik 40,3 persen pada semester I</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 19:20:34 +0700</t>
+          <t>Fri, 31 Jul 2026 19:23:27 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PT Bank Neo Commerce Tbk (BNC) membukukan laba bersih setelah pajak (profit after tax/PAT) sebesar Rp294,85 miliar pada ...</t>
+          <t>PT Bank SMBC Indonesia Tbk membukukan laba bersih setelah pajak konsolidasi yang diatribusikan kepada pemilik entitas ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674772/bank-neo-commerce-bukukan-laba-bersih-rp29485-m-pada-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5674780/laba-konsolidasi-bank-smbc-indonesia-naik-403-persen-pada-semester-i</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/WhatsApp-Image-2026-07-31-at-17.22.56.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/Foto-2-3.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-04 01:54 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-31.xlsx
+++ b/data/berita_antara_2026-07-31.xlsx
@@ -768,33 +768,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
+          <t>IIF bukukan aset Rp15 triliun dan pembiayaan baru Rp2,5 triliun</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
+          <t>Fri, 31 Jul 2026 23:05:50 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
+          <t>PT Indonesia Infrastructure Finance (IIF) mencatat aset Rp15 triliun dan komitmen pembiayaan baru Rp2,5 triliun pada ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
+          <t>https://www.antaranews.com/berita/5675203/iif-bukukan-aset-rp15-triliun-dan-pembiayaan-baru-rp25-triliun</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/B9A16C4E-32D5-4162-BA5C-89F5A5135BC8.jpeg</t>
         </is>
       </c>
     </row>
@@ -806,61 +806,61 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
+          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
+          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
+          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
+          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IIF bukukan aset Rp15 triliun dan pembiayaan baru Rp2,5 triliun</t>
+          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 23:05:50 +0700</t>
+          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PT Indonesia Infrastructure Finance (IIF) mencatat aset Rp15 triliun dan komitmen pembiayaan baru Rp2,5 triliun pada ...</t>
+          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675203/iif-bukukan-aset-rp15-triliun-dan-pembiayaan-baru-rp25-triliun</t>
+          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/B9A16C4E-32D5-4162-BA5C-89F5A5135BC8.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-04 15:14 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-31.xlsx
+++ b/data/berita_antara_2026-07-31.xlsx
@@ -817,33 +817,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
+          <t>IHSG Jumat dibuka menguat 33,26 poin ke posisi 6.219</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
+          <t>Fri, 31 Jul 2026 09:12:28 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat pagi dibuka menguat 33,26 poin atau 0,54 ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
+          <t>https://www.antaranews.com/berita/5673745/ihsg-jumat-dibuka-menguat-3326-poin-ke-posisi-6219</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-02.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -860,28 +860,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
+          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
+          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
+          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
+          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -893,33 +893,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IHSG jelang akhir pekan ditutup menguat ikuti bursa kawasan Asia</t>
+          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 17:03:08 +0700</t>
+          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat sore, ditutup naik mengikuti penguatan bursa ...</t>
+          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674467/ihsg-jelang-akhir-pekan-ditutup-menguat-ikuti-bursa-kawasan-asia</t>
+          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828639.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -936,28 +936,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Analis: Kinerja keuangan tentukan arah pergerakan saham pertambangan</t>
+          <t>IHSG jelang akhir pekan ditutup menguat ikuti bursa kawasan Asia</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 16:00:07 +0700</t>
+          <t>Fri, 31 Jul 2026 17:03:08 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Market Analyst Mirae Asset Sekuritas Indonesia, Nafan Aji Gusta menyampaikan bahwa kinerja laporan keuangan ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat sore, ditutup naik mengikuti penguatan bursa ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674312/analis-kinerja-keuangan-tentukan-arah-pergerakan-saham-pertambangan</t>
+          <t>https://www.antaranews.com/berita/5674467/ihsg-jelang-akhir-pekan-ditutup-menguat-ikuti-bursa-kawasan-asia</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/ihsg-ditutup-anjlok-pada-pekan-ketiga-mei-2026-2790781.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828639.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -974,28 +974,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PLN UID Sulselrabar resmikan "HSSE control center" perkuat keselamatan</t>
+          <t>Analis: Kinerja keuangan tentukan arah pergerakan saham pertambangan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 10:23:03 +0700</t>
+          <t>Fri, 31 Jul 2026 16:00:07 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PT PLN Unit Induk Distribusi Sulawesi Selatan, Sulawesi Tenggara dan Sulawesi Barat (UID Sulselrabar) meresmikan ...</t>
+          <t>Senior Market Analyst Mirae Asset Sekuritas Indonesia, Nafan Aji Gusta menyampaikan bahwa kinerja laporan keuangan ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673821/pln-uid-sulselrabar-resmikan-hsse-control-center-perkuat-keselamatan</t>
+          <t>https://www.antaranews.com/berita/5674312/analis-kinerja-keuangan-tentukan-arah-pergerakan-saham-pertambangan</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1002890680.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/ihsg-ditutup-anjlok-pada-pekan-ketiga-mei-2026-2790781.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1012,28 +1012,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IHSG menguat ikuti bursa kawasan Asia dan global</t>
+          <t>PLN UID Sulselrabar resmikan "HSSE control center" perkuat keselamatan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 09:38:38 +0700</t>
+          <t>Fri, 31 Jul 2026 10:23:03 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat bergerak naik mengikuti penguatan bursa saham ...</t>
+          <t>PT PLN Unit Induk Distribusi Sulawesi Selatan, Sulawesi Tenggara dan Sulawesi Barat (UID Sulselrabar) meresmikan ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673777/ihsg-menguat-ikuti-bursa-kawasan-asia-dan-global</t>
+          <t>https://www.antaranews.com/berita/5673821/pln-uid-sulselrabar-resmikan-hsse-control-center-perkuat-keselamatan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1002890680.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1050,28 +1050,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IHSG Jumat dibuka menguat 33,26 poin ke posisi 6.219</t>
+          <t>IHSG menguat ikuti bursa kawasan Asia dan global</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 09:12:28 +0700</t>
+          <t>Fri, 31 Jul 2026 09:38:38 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat pagi dibuka menguat 33,26 poin atau 0,54 ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat bergerak naik mengikuti penguatan bursa saham ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673745/ihsg-jumat-dibuka-menguat-3326-poin-ke-posisi-6219</t>
+          <t>https://www.antaranews.com/berita/5673777/ihsg-menguat-ikuti-bursa-kawasan-asia-dan-global</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-02.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">

</xml_diff>

<commit_message>
Update berita 2026-08-05 03:44 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-31.xlsx
+++ b/data/berita_antara_2026-07-31.xlsx
@@ -855,33 +855,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
+          <t>PLN UID Sulselrabar resmikan "HSSE control center" perkuat keselamatan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
+          <t>Fri, 31 Jul 2026 10:23:03 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
+          <t>PT PLN Unit Induk Distribusi Sulawesi Selatan, Sulawesi Tenggara dan Sulawesi Barat (UID Sulselrabar) meresmikan ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
+          <t>https://www.antaranews.com/berita/5673821/pln-uid-sulselrabar-resmikan-hsse-control-center-perkuat-keselamatan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1002890680.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -893,33 +893,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
+          <t>IHSG menguat ikuti bursa kawasan Asia dan global</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
+          <t>Fri, 31 Jul 2026 09:38:38 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat bergerak naik mengikuti penguatan bursa saham ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
+          <t>https://www.antaranews.com/berita/5673777/ihsg-menguat-ikuti-bursa-kawasan-asia-dan-global</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -931,33 +931,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IHSG jelang akhir pekan ditutup menguat ikuti bursa kawasan Asia</t>
+          <t>Cara war tiket upacara 17 Agustus 2026 di Istana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 17:03:08 +0700</t>
+          <t>Fri, 31 Jul 2026 15:15:56 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat sore, ditutup naik mengikuti penguatan bursa ...</t>
+          <t>Masyarakat yang ingin mengikuti upacara peringatan HUT ke-81 Kemerdekaan Republik Indonesia di Istana Merdeka pada 17 ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674467/ihsg-jelang-akhir-pekan-ditutup-menguat-ikuti-bursa-kawasan-asia</t>
+          <t>https://www.antaranews.com/berita/5674240/cara-war-tiket-upacara-17-agustus-2026-di-istana</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828639.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/18/193.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -969,33 +969,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Analis: Kinerja keuangan tentukan arah pergerakan saham pertambangan</t>
+          <t>HUT RI 2026: Tema, logo resmi, makna, dan jadwal upacara 17 Agustus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 16:00:07 +0700</t>
+          <t>Fri, 31 Jul 2026 13:39:10 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Market Analyst Mirae Asset Sekuritas Indonesia, Nafan Aji Gusta menyampaikan bahwa kinerja laporan keuangan ...</t>
+          <t>Indonesia akan memperingati Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026. ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5674312/analis-kinerja-keuangan-tentukan-arah-pergerakan-saham-pertambangan</t>
+          <t>https://www.antaranews.com/berita/5674081/hut-ri-2026-tema-logo-resmi-makna-dan-jadwal-upacara-17-agustus</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/ihsg-ditutup-anjlok-pada-pekan-ketiga-mei-2026-2790781.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000032945.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1012,28 +1012,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PLN UID Sulselrabar resmikan "HSSE control center" perkuat keselamatan</t>
+          <t>IHSG jelang akhir pekan ditutup menguat ikuti bursa kawasan Asia</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 10:23:03 +0700</t>
+          <t>Fri, 31 Jul 2026 17:03:08 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PT PLN Unit Induk Distribusi Sulawesi Selatan, Sulawesi Tenggara dan Sulawesi Barat (UID Sulselrabar) meresmikan ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat sore, ditutup naik mengikuti penguatan bursa ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673821/pln-uid-sulselrabar-resmikan-hsse-control-center-perkuat-keselamatan</t>
+          <t>https://www.antaranews.com/berita/5674467/ihsg-jelang-akhir-pekan-ditutup-menguat-ikuti-bursa-kawasan-asia</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/1002890680.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828639.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1050,28 +1050,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IHSG menguat ikuti bursa kawasan Asia dan global</t>
+          <t>Analis: Kinerja keuangan tentukan arah pergerakan saham pertambangan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 31 Jul 2026 09:38:38 +0700</t>
+          <t>Fri, 31 Jul 2026 16:00:07 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Jumat bergerak naik mengikuti penguatan bursa saham ...</t>
+          <t>Senior Market Analyst Mirae Asset Sekuritas Indonesia, Nafan Aji Gusta menyampaikan bahwa kinerja laporan keuangan ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5673777/ihsg-menguat-ikuti-bursa-kawasan-asia-dan-global</t>
+          <t>https://www.antaranews.com/berita/5674312/analis-kinerja-keuangan-tentukan-arah-pergerakan-saham-pertambangan</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-05.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/ihsg-ditutup-anjlok-pada-pekan-ketiga-mei-2026-2790781.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">

</xml_diff>